<commit_message>
feat(nepool): Cloud Capture as primary capture path + onboarding redo
Replace extension-first NEPOOL onboarding with Array Operator-style dual path:
Cloud Capture recommended (store utility logins server-side; harvester pulls
bills 24/7), extension kept as private fallback. Always-on (no feature flag).

- Account: mode-aware CloudCaptureCard vault (honest login vs scrape status)
  + capture_mode toggle; extension PortalAccessCard for device/legacy tenants
- Dashboard: suppress stale-extension banner when capture_mode=cloud
- Onboarding: Connect fork → CloudConnect (early complete + vault) or Extension
- GetStarted/Welcome/privacy: cloud-first narrative; dual-mode consent
- Support map: NEPOOL cloud default + wizard path notes
- Rebuild api/app_dist + api/onboarding_dist (committed SPA bundles)

No backend API changes — /v1/cloud-capture/* and harvester already live.
No forced migration of existing extension operators.
</commit_message>
<xml_diff>
--- a/api/onboarding_dist/sample.xlsx
+++ b/api/onboarding_dist/sample.xlsx
@@ -509,229 +509,229 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Q1 2025</t>
+          <t>Q4 2024</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>16.4</v>
+        <v>23.2</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>16.4</v>
+        <v>23.2</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="4" t="n">
-        <v>22.2</v>
+        <v>15.5</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>22.2</v>
+        <v>15.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q1 2025</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>24.3</v>
+        <v>16.4</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>24.3</v>
+        <v>16.4</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="n">
-        <v>28.2</v>
+        <v>18.3</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>28.2</v>
+        <v>18.3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="n">
-        <v>32.6</v>
+        <v>22.2</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>32.6</v>
+        <v>22.2</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Q2 2025</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>34</v>
+        <v>24.3</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>34</v>
+        <v>24.3</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="4" t="n">
-        <v>32.4</v>
+        <v>28.2</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>32.4</v>
+        <v>28.2</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="4" t="n">
-        <v>28.8</v>
+        <v>32.6</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>28.8</v>
+        <v>32.6</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Q3 2025</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>25.2</v>
+        <v>34</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>25.2</v>
+        <v>34</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="n">
-        <v>18.3</v>
+        <v>32.4</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>18.3</v>
+        <v>32.4</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="n">
-        <v>15</v>
+        <v>28.8</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>15</v>
+        <v>28.8</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Q1 2026</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>15.6</v>
+        <v>25.2</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>15.6</v>
+        <v>25.2</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="4" t="n">
-        <v>17.5</v>
+        <v>18.3</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>17.5</v>
+        <v>18.3</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="4" t="n">
-        <v>21.4</v>
+        <v>15</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>21.4</v>
+        <v>15</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q1 2026</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>26.3</v>
+        <v>15.6</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>26.3</v>
+        <v>15.6</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="4" t="n">
-        <v>30.2</v>
+        <v>17.5</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>30.2</v>
+        <v>17.5</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="4" t="n">
-        <v>31.8</v>
+        <v>21.4</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>31.8</v>
+        <v>21.4</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31">
@@ -797,229 +797,229 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Q1 2025</t>
+          <t>Q4 2024</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>19.65</v>
+        <v>26.45</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>19.65</v>
+        <v>26.45</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="n">
-        <v>21.55</v>
+        <v>22.35</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>21.55</v>
+        <v>22.35</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="4" t="n">
-        <v>25.45</v>
+        <v>18.75</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>25.45</v>
+        <v>18.75</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Q2 2025</t>
+          <t>Q1 2025</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>27.55</v>
+        <v>19.65</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>27.55</v>
+        <v>19.65</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="n">
-        <v>31.45</v>
+        <v>21.55</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>31.45</v>
+        <v>21.55</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="n">
-        <v>35</v>
+        <v>25.45</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>35</v>
+        <v>25.45</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Q3 2025</t>
+          <t>Q2 2025</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>35</v>
+        <v>27.55</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>35</v>
+        <v>27.55</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="4" t="n">
-        <v>35</v>
+        <v>31.45</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>35</v>
+        <v>31.45</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="4" t="n">
-        <v>32.05</v>
+        <v>35</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>32.05</v>
+        <v>35</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Q4 2025</t>
+          <t>Q3 2025</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>28.45</v>
+        <v>35</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>28.45</v>
+        <v>35</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="n">
-        <v>21.55</v>
+        <v>35</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>21.55</v>
+        <v>35</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="n">
-        <v>17.95</v>
+        <v>32.05</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>17.95</v>
+        <v>32.05</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>17</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Q1 2026</t>
+          <t>Q4 2025</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>18.85</v>
+        <v>28.45</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>18.85</v>
+        <v>28.45</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="4" t="n">
-        <v>20.75</v>
+        <v>21.55</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>20.75</v>
+        <v>21.55</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="4" t="n">
-        <v>24.65</v>
+        <v>17.95</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>24.65</v>
+        <v>17.95</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Q2 2026</t>
+          <t>Q1 2026</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>29.55</v>
+        <v>18.85</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>29.55</v>
+        <v>18.85</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="4" t="n">
-        <v>33.45</v>
+        <v>20.75</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>33.45</v>
+        <v>20.75</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="4" t="n">
-        <v>35</v>
+        <v>24.65</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>35</v>
+        <v>24.65</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31">

</xml_diff>